<commit_message>
Restructure task sheet: Location vs Brand (Umami=brand @ Central 50)
</commit_message>
<xml_diff>
--- a/Task_Sheet_List.xlsx
+++ b/Task_Sheet_List.xlsx
@@ -41,15 +41,15 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,12 +63,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDF2E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF1FB"/>
+        <fgColor rgb="00E9F7EF"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -107,22 +112,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -493,8 +507,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -546,527 +560,527 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Umami</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>10 inch glass partition</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Shelf</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Work table</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Cash drawer missing</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Power load increase 21 kwatt</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>2 power point</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>AC and cooling solution</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Logo colour need to change</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Top logo</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr"/>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>District 9</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Need to have separate sitting space for staff</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Need to cover by making waterproof cover</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="inlineStr"/>
-      <c r="B13" s="7" t="inlineStr"/>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Brand signage should be proper lit</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>No space for keeping cushion and chairs in the rain</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr"/>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Garbage drum should be painted every month</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Mist</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Central 50</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Need to cover by making waterproof cover</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Cameras</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>No space for keeping cushion and chairs in the rain</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Camera connectors in the kiosks</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Mist</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Digital menu connectors</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Cameras</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Extension board 5</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Camera connectors in the kiosks</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Floor scrubbing machine required</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="3" t="inlineStr"/>
-      <c r="B20" s="4" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Digital menu connectors</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Garbage drum needs wheels installed underneath</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Extension board 5</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Furniture rope needs to fix</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Floor scrubbing machine required</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>One more house keeping guy</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Garbage drum needs wheels installed underneath</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Plants for ETL drum signage</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="3" t="inlineStr"/>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Furniture rope needs to fix</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>RO for mist</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="3" t="inlineStr"/>
-      <c r="B25" s="4" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>One more house keeping guy</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>The drawer should be covered with the lid</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Plants for ETL drum signage</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>District 9</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Need to have separate sitting space for staff</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="3" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>RO for mist</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
+      <c r="A27" s="6" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Brand signage should be proper lit</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="3" t="inlineStr"/>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>The drawer should be covered with the lid</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
+      <c r="A28" s="6" t="inlineStr"/>
+      <c r="B28" s="6" t="inlineStr"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Garbage drum should be painted every month</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="6" t="inlineStr"/>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Bennett University</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Store need to be vacated</t>
         </is>
       </c>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="6" t="inlineStr"/>
-      <c r="B30" s="7" t="inlineStr"/>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr"/>
+      <c r="B30" s="9" t="inlineStr"/>
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>Store needs extra electrical point</t>
         </is>
       </c>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="6" t="inlineStr"/>
-      <c r="B31" s="7" t="inlineStr"/>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr"/>
+      <c r="B31" s="9" t="inlineStr"/>
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>More furniture required</t>
         </is>
       </c>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="6" t="inlineStr"/>
-      <c r="B32" s="7" t="inlineStr"/>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr"/>
+      <c r="B32" s="9" t="inlineStr"/>
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>Water between store and truck</t>
         </is>
       </c>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="6" t="inlineStr"/>
-      <c r="B33" s="7" t="inlineStr"/>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr"/>
+      <c r="B33" s="9" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Wi-Fi connection for eggspert</t>
         </is>
       </c>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="6" t="inlineStr"/>
-      <c r="B34" s="7" t="inlineStr"/>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr"/>
+      <c r="B34" s="9" t="inlineStr"/>
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>House keeping staff uniforms</t>
         </is>
       </c>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="6" t="inlineStr"/>
-      <c r="B35" s="7" t="inlineStr"/>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr"/>
+      <c r="B35" s="9" t="inlineStr"/>
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>B2B menu board</t>
         </is>
       </c>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="6" t="inlineStr"/>
-      <c r="B36" s="7" t="inlineStr"/>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="A36" s="9" t="inlineStr"/>
+      <c r="B36" s="9" t="inlineStr"/>
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Signage light</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="6" t="inlineStr"/>
-      <c r="B37" s="7" t="inlineStr"/>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr"/>
+      <c r="B37" s="9" t="inlineStr"/>
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>Ducting</t>
         </is>
       </c>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="6" t="inlineStr"/>
-      <c r="B38" s="7" t="inlineStr"/>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="A38" s="9" t="inlineStr"/>
+      <c r="B38" s="9" t="inlineStr"/>
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>First aid kit for every truck</t>
         </is>
       </c>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="6" t="inlineStr"/>
-      <c r="B39" s="7" t="inlineStr"/>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr"/>
+      <c r="B39" s="9" t="inlineStr"/>
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Fire blanket</t>
         </is>
       </c>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="6" t="inlineStr"/>
-      <c r="B40" s="7" t="inlineStr"/>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="A40" s="9" t="inlineStr"/>
+      <c r="B40" s="9" t="inlineStr"/>
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>Fire extinguisher for electrical and oil</t>
         </is>
       </c>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="6" t="inlineStr"/>
-      <c r="B41" s="7" t="inlineStr"/>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="A41" s="9" t="inlineStr"/>
+      <c r="B41" s="9" t="inlineStr"/>
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Rubber shoes for tables</t>
         </is>
       </c>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Increase row height for easier hand-writing
</commit_message>
<xml_diff>
--- a/Task_Sheet_List.xlsx
+++ b/Task_Sheet_List.xlsx
@@ -559,7 +559,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Central 50</t>
@@ -580,7 +580,7 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr"/>
       <c r="C4" s="4" t="inlineStr">
@@ -593,7 +593,7 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr"/>
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr">
@@ -606,7 +606,7 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr"/>
       <c r="C6" s="4" t="inlineStr">
@@ -619,7 +619,7 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr"/>
       <c r="B7" s="3" t="inlineStr"/>
       <c r="C7" s="4" t="inlineStr">
@@ -632,7 +632,7 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="3" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr"/>
       <c r="C8" s="4" t="inlineStr">
@@ -645,7 +645,7 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
       <c r="B9" s="3" t="inlineStr"/>
       <c r="C9" s="4" t="inlineStr">
@@ -658,7 +658,7 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="3" t="inlineStr"/>
       <c r="B10" s="3" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr">
@@ -671,7 +671,7 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr"/>
       <c r="B11" s="3" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr">
@@ -684,7 +684,7 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="3" t="inlineStr"/>
       <c r="B12" s="3" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr">
@@ -697,7 +697,7 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr"/>
       <c r="B13" s="3" t="inlineStr"/>
       <c r="C13" s="4" t="inlineStr">
@@ -710,7 +710,7 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="3" t="inlineStr"/>
       <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="4" t="inlineStr">
@@ -723,7 +723,7 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr"/>
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" s="3" t="inlineStr"/>
       <c r="B16" s="3" t="inlineStr"/>
       <c r="C16" s="4" t="inlineStr">
@@ -749,7 +749,7 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="3" t="inlineStr"/>
       <c r="B17" s="3" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr">
@@ -762,7 +762,7 @@
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" s="3" t="inlineStr"/>
       <c r="B18" s="3" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr">
@@ -775,7 +775,7 @@
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="42" customHeight="1">
       <c r="A19" s="3" t="inlineStr"/>
       <c r="B19" s="3" t="inlineStr"/>
       <c r="C19" s="4" t="inlineStr">
@@ -788,7 +788,7 @@
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="3" t="inlineStr"/>
       <c r="B20" s="3" t="inlineStr"/>
       <c r="C20" s="4" t="inlineStr">
@@ -801,7 +801,7 @@
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" s="3" t="inlineStr"/>
       <c r="B21" s="3" t="inlineStr"/>
       <c r="C21" s="4" t="inlineStr">
@@ -814,7 +814,7 @@
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="3" t="inlineStr"/>
       <c r="B22" s="3" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr">
@@ -827,7 +827,7 @@
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="3" t="inlineStr"/>
       <c r="B23" s="3" t="inlineStr"/>
       <c r="C23" s="4" t="inlineStr">
@@ -840,7 +840,7 @@
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="42" customHeight="1">
       <c r="A24" s="3" t="inlineStr"/>
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="4" t="inlineStr">
@@ -853,7 +853,7 @@
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="3" t="inlineStr"/>
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr">
@@ -866,7 +866,7 @@
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>District 9</t>
@@ -883,7 +883,7 @@
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="6" t="inlineStr"/>
       <c r="B27" s="6" t="inlineStr"/>
       <c r="C27" s="7" t="inlineStr">
@@ -896,7 +896,7 @@
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="6" t="inlineStr"/>
       <c r="B28" s="6" t="inlineStr"/>
       <c r="C28" s="7" t="inlineStr">
@@ -909,7 +909,7 @@
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="42" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Bennett University</t>
@@ -926,7 +926,7 @@
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
     </row>
-    <row r="30" ht="30" customHeight="1">
+    <row r="30" ht="42" customHeight="1">
       <c r="A30" s="9" t="inlineStr"/>
       <c r="B30" s="9" t="inlineStr"/>
       <c r="C30" s="10" t="inlineStr">
@@ -939,7 +939,7 @@
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="42" customHeight="1">
       <c r="A31" s="9" t="inlineStr"/>
       <c r="B31" s="9" t="inlineStr"/>
       <c r="C31" s="10" t="inlineStr">
@@ -952,7 +952,7 @@
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" s="9" t="inlineStr"/>
       <c r="B32" s="9" t="inlineStr"/>
       <c r="C32" s="10" t="inlineStr">
@@ -965,7 +965,7 @@
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" s="9" t="inlineStr"/>
       <c r="B33" s="9" t="inlineStr"/>
       <c r="C33" s="10" t="inlineStr">
@@ -978,7 +978,7 @@
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
     </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" s="9" t="inlineStr"/>
       <c r="B34" s="9" t="inlineStr"/>
       <c r="C34" s="10" t="inlineStr">
@@ -991,7 +991,7 @@
       <c r="F34" s="11" t="n"/>
       <c r="G34" s="11" t="n"/>
     </row>
-    <row r="35" ht="30" customHeight="1">
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" s="9" t="inlineStr"/>
       <c r="B35" s="9" t="inlineStr"/>
       <c r="C35" s="10" t="inlineStr">
@@ -1004,7 +1004,7 @@
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" s="9" t="inlineStr"/>
       <c r="B36" s="9" t="inlineStr"/>
       <c r="C36" s="10" t="inlineStr">
@@ -1017,7 +1017,7 @@
       <c r="F36" s="11" t="n"/>
       <c r="G36" s="11" t="n"/>
     </row>
-    <row r="37" ht="30" customHeight="1">
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" s="9" t="inlineStr"/>
       <c r="B37" s="9" t="inlineStr"/>
       <c r="C37" s="10" t="inlineStr">
@@ -1030,7 +1030,7 @@
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" s="9" t="inlineStr"/>
       <c r="B38" s="9" t="inlineStr"/>
       <c r="C38" s="10" t="inlineStr">
@@ -1043,7 +1043,7 @@
       <c r="F38" s="11" t="n"/>
       <c r="G38" s="11" t="n"/>
     </row>
-    <row r="39" ht="30" customHeight="1">
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" s="9" t="inlineStr"/>
       <c r="B39" s="9" t="inlineStr"/>
       <c r="C39" s="10" t="inlineStr">
@@ -1056,7 +1056,7 @@
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
     </row>
-    <row r="40" ht="30" customHeight="1">
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" s="9" t="inlineStr"/>
       <c r="B40" s="9" t="inlineStr"/>
       <c r="C40" s="10" t="inlineStr">
@@ -1069,7 +1069,7 @@
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="11" t="n"/>
     </row>
-    <row r="41" ht="30" customHeight="1">
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" s="9" t="inlineStr"/>
       <c r="B41" s="9" t="inlineStr"/>
       <c r="C41" s="10" t="inlineStr">

</xml_diff>